<commit_message>
feat(mockup): close Phase 5 portfolio and capacity planning
</commit_message>
<xml_diff>
--- a/04_Developement_tracking/Mini_Rally_Product_Plan.xlsx
+++ b/04_Developement_tracking/Mini_Rally_Product_Plan.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra109800aecf940a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="2" r:id="R24891df4abb545a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BA Tasks" sheetId="3" r:id="R48e3900e9ae14292"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEV Tasks" sheetId="4" r:id="R3312ad1c136040ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="5" r:id="R54c293758b8e43a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc4d4e13c9aa94da6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Roadmap" sheetId="2" r:id="R8c9eb6e2538346b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BA Tasks" sheetId="3" r:id="R2a26c085553640bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEV Tasks" sheetId="4" r:id="R0447679099534b5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="5" r:id="R125ffe1788d448b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -769,10 +769,8 @@
       </x:c>
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
-      <x:c r="A2" s="6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Single planning workbook | Baseline: 2026-07-26 | Scope: BA, FE DEV, DevInt and UAT through Phase 5</x:t>
-        </x:is>
+      <x:c r="A2" s="6" t="str">
+        <x:v>Single planning workbook | Baseline: 2026-07-28 | Scope: BA, FE DEV, DevInt and UAT through closed Phase 5</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26" customHeight="1">
@@ -816,10 +814,8 @@
           <x:t xml:space="preserve">BA baseline</x:t>
         </x:is>
       </x:c>
-      <x:c r="H5" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phase 0-5 governance aligned</x:t>
-        </x:is>
+      <x:c r="H5" s="15" t="str">
+        <x:v>Phase 0-5 BA baseline aligned; Phase 5 DEV handoff ready</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -829,7 +825,7 @@
         </x:is>
       </x:c>
       <x:c r="B6" s="15" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D6" s="15" t="inlineStr">
         <x:is>
@@ -845,10 +841,8 @@
           <x:t xml:space="preserve">DEV current</x:t>
         </x:is>
       </x:c>
-      <x:c r="H6" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phase 0-4 DevInt; Phase 5 production not started</x:t>
-        </x:is>
+      <x:c r="H6" s="15" t="str">
+        <x:v>Phase 0-4 DevInt active; Phase 5 production not started</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -858,7 +852,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="15" t="n">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D7" s="15" t="inlineStr">
         <x:is>
@@ -875,7 +869,7 @@
         </x:is>
       </x:c>
       <x:c r="H7" s="15" t="str">
-        <x:v>P5.2 Capacity Planning active; docs aligned and mockup implementation next</x:v>
+        <x:v>Start Phase 5 production analysis from dedicated DEV handoff</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -888,9 +882,10 @@
     <x:row r="10">
       <x:c r="A10" s="66" t="str">
         <x:v>1. BA owns business rules, SRS/mockup alignment and acceptance.
-2. Every Phase 5 feature follows: propose -&gt; BA confirm -&gt; docs align -&gt; implement -&gt; verify -&gt; BA accept -&gt; close.
-3. BA/Mockup readiness and Production readiness are always separate.
-4. Phase 5 closes only after P5.1-P5.3 close, tests/traceability pass and BA accepts; only then create the Phase 5 DEV handoff.</x:v>
+2. Closed Phase 5 scope is Portfolio Items plus Capacity Planning.
+3. Release Planning and Release Tracking are excluded; Reports are Future Backlog only.
+4. BA/Mockup readiness, DEV handoff readiness and Production readiness remain separate.
+5. Future changes require propose -&gt; BA confirm -&gt; docs -&gt; implement -&gt; verify -&gt; accept.</x:v>
       </x:c>
       <x:c r="B10" s="67" t="n"/>
       <x:c r="C10" s="67" t="n"/>
@@ -928,39 +923,37 @@
     </x:row>
     <x:row r="16" ht="32" customHeight="1">
       <x:c r="A16" s="11" t="str">
-        <x:v>Phase 5 Order</x:v>
-      </x:c>
-      <x:c r="B16" s="11" t="n">
+        <x:v>Phase 5 Closed</x:v>
+      </x:c>
+      <x:c r="B16" s="11" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C16" s="11" t="str">
         <x:v>P5.0 Rebaseline</x:v>
       </x:c>
-      <x:c r="D16" s="11" t="n">
+      <x:c r="D16" s="11" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="E16" s="11" t="str">
-        <x:v>P5.1 Closure</x:v>
-      </x:c>
-      <x:c r="F16" s="11" t="n">
+        <x:v>P5.1 Portfolio Items</x:v>
+      </x:c>
+      <x:c r="F16" s="11" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="G16" s="11" t="str">
-        <x:v>P5.2 Capacity -&gt; P5.3 Tracking</x:v>
-      </x:c>
-      <x:c r="H16" s="11" t="n">
+        <x:v>P5.2 Capacity Planning</x:v>
+      </x:c>
+      <x:c r="H16" s="11" t="str">
         <x:v>4</x:v>
       </x:c>
       <x:c r="I16" s="11" t="str">
-        <x:v>P5.4 Closeout</x:v>
+        <x:v>P5.3 removed / P5.4 DEV Handoff</x:v>
       </x:c>
       <x:c r="J16" s="11" t="n"/>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
-      <x:c r="A18" s="52" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Sources of truth: RECONCILED_SOURCE_OF_TRUTH.md, Phase 5/PHASE5_DEVELOPMENT_TRACKING.md, phase SRS/checklists, 06_Dev testing align and 07_Test Business/specs. The Phase 5 DEV handoff is created only after phase close.</x:t>
-        </x:is>
+      <x:c r="A18" s="52" t="str">
+        <x:v>Sources of truth: RECONCILED_SOURCE_OF_TRUTH.md, Phase 5/PHASE5_DEV_HANDOFF.md, Phase 5 SRS/catalogs, PHASE5_DEVELOPMENT_TRACKING.md and 07_Test Business/specs. Phase 5 is BA/mockup closed; production implementation is not started.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1003,7 +996,7 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Product baseline 2026-07-26 | P5-GOV v2 confirmed; DEV dates remain an editable proposal</x:v>
+        <x:v>Product baseline 2026-07-28 | P5-GOV v4 closed; DEV dates remain an editable proposal</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="32" customHeight="1">
@@ -1298,26 +1291,28 @@
         </x:is>
       </x:c>
       <x:c r="C10" s="15" t="str">
-        <x:v>Portfolio Items, Capacity Planning and Release Tracking; Release Planning deferred</x:v>
+        <x:v>Portfolio Items and Capacity Planning; Release Planning/Tracking excluded</x:v>
       </x:c>
       <x:c r="D10" s="22" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="E10" s="34" t="str">
-        <x:v>Needs BA</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="F10" s="15" t="str">
-        <x:v>P5.2 Capacity Planning</x:v>
+        <x:v>DEV Handoff</x:v>
       </x:c>
       <x:c r="G10" s="74" t="n">
         <x:v>46229</x:v>
       </x:c>
-      <x:c r="H10" s="74"/>
+      <x:c r="H10" s="74" t="n">
+        <x:v>46231</x:v>
+      </x:c>
       <x:c r="I10" s="15" t="str">
-        <x:v>P5.1-P5.3 BA accepted; Phase 5 tests and traceability complete; Phase 5 DEV handoff created</x:v>
+        <x:v>P5.1/P5.2 BA accepted; scope/tests/workbook reconciled; Phase 5 DEV handoff created</x:v>
       </x:c>
       <x:c r="J10" s="15" t="str">
-        <x:v>Implement P5.2 Capacity Planning after docs alignment</x:v>
+        <x:v>Start production analysis from Phase 5 DEV handoff</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="58" customHeight="1">
@@ -1332,7 +1327,7 @@
         </x:is>
       </x:c>
       <x:c r="C11" s="15" t="str">
-        <x:v>Team/Iteration boards, generic Reports, Theme/Initiative, Release Planning, burnup history and multi-Release scenarios</x:v>
+        <x:v>Team/Iteration boards, Reports, Release Planning, Release Tracking, Theme/deeper hierarchy, burnup history and multi-Release scenarios</x:v>
       </x:c>
       <x:c r="D11" s="25" t="str">
         <x:v>Future Backlog</x:v>
@@ -2990,10 +2985,8 @@
       </x:c>
     </x:row>
     <x:row r="28" ht="94.5" customHeight="1">
-      <x:c r="A28" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BA-0501</x:t>
-        </x:is>
+      <x:c r="A28" s="15" t="str">
+        <x:v>BA-0501</x:v>
       </x:c>
       <x:c r="B28" s="15" t="inlineStr">
         <x:is>
@@ -3036,143 +3029,105 @@
       <x:c r="J28" s="74" t="n">
         <x:v>46229</x:v>
       </x:c>
-      <x:c r="K28" s="74" t="n"/>
+      <x:c r="K28" s="74" t="n">
+        <x:v>46231</x:v>
+      </x:c>
       <x:c r="L28" s="76" t="str">
-        <x:v>P5.1 Amendment v3 implementation verified and BA accepted; continue Phase 5</x:v>
+        <x:v>Feature and Epic flows, formulas, archive rules and accepted UI are documented and BA accepted</x:v>
       </x:c>
       <x:c r="M28" s="76" t="str">
-        <x:v>BA accepted 2026-07-26</x:v>
+        <x:v>DEV handoff</x:v>
       </x:c>
       <x:c r="N28" s="76" t="str">
-        <x:v>P5.1 plus BA-confirmed Amendment v3 accepted 2026-07-26: shared Feature-linked Work Item flow, Backlog shows Unscheduled only, Task Estimate/To Do/Actual independent with complete setting To Do to 0. Build and runtime smoke completed; close P5.1 and continue Phase 5. Production API/persistence remains dev scope.</x:v>
+        <x:v>P5.1 Feature baseline and Epic amendment closed 2026-07-28; production persistence/API/RBAC remains DEV scope</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="54" customHeight="1">
-      <x:c r="A29" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BA-0502</x:t>
-        </x:is>
+      <x:c r="A29" s="15" t="str">
+        <x:v>BA-F501</x:v>
       </x:c>
       <x:c r="B29" s="15" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Phase 5</x:t>
         </x:is>
       </x:c>
-      <x:c r="C29" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Release Planning</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D29" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Define and accept Feature-to-Release planning board</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E29" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phase 5/02_Release_Planning/SRS.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F29" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BA-0501</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G29" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H29" s="22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planned</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I29" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BA/PO</x:t>
-        </x:is>
+      <x:c r="C29" s="15" t="str">
+        <x:v>Release Planning</x:v>
+      </x:c>
+      <x:c r="D29" s="15" t="str">
+        <x:v>Keep Release Planning outside the closed Phase 5 MVP</x:v>
+      </x:c>
+      <x:c r="E29" s="15" t="str">
+        <x:v>Future_Backlog</x:v>
+      </x:c>
+      <x:c r="F29" s="15" t="str">
+        <x:v>BA decision 2026-07-26</x:v>
+      </x:c>
+      <x:c r="G29" s="15" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="H29" s="22" t="str">
+        <x:v>Future Backlog</x:v>
+      </x:c>
+      <x:c r="I29" s="15" t="str">
+        <x:v>BA/PO</x:v>
       </x:c>
       <x:c r="J29" s="74" t="n"/>
       <x:c r="K29" s="74" t="n"/>
-      <x:c r="L29" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Assign, move and unassign Features without duplicating Release management</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M29" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Feature proposal</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N29" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Starts only after P5.1 closes</x:t>
-        </x:is>
+      <x:c r="L29" s="15" t="str">
+        <x:v>No Release Planning behavior is required for Phase 5 close</x:v>
+      </x:c>
+      <x:c r="M29" s="15" t="str">
+        <x:v>Future backlog review</x:v>
+      </x:c>
+      <x:c r="N29" s="15" t="str">
+        <x:v>Capacity Planning publish is the accepted Phase 5 planning action</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
-      <x:c r="A30" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BA-0503</x:t>
-        </x:is>
+      <x:c r="A30" s="15" t="str">
+        <x:v>BA-F502</x:v>
       </x:c>
       <x:c r="B30" s="15" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Phase 5</x:t>
         </x:is>
       </x:c>
-      <x:c r="C30" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Release Tracking</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D30" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Define and accept Release KPI and Feature progress tracking</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E30" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phase 5/03_Release_Tracking/SRS.md</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F30" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BA-0502</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G30" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H30" s="22" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Planned</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I30" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BA/PO</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J30" s="74" t="n"/>
-      <x:c r="K30" s="74" t="n"/>
-      <x:c r="L30" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Plan Estimate rollup, zero-estimate handling and no auto Release state pass UAT</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M30" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Feature proposal</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N30" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Burnup waits for trustworthy history</x:t>
-        </x:is>
+      <x:c r="C30" s="15" t="str">
+        <x:v>Release Tracking</x:v>
+      </x:c>
+      <x:c r="D30" s="15" t="str">
+        <x:v>Remove dedicated Release Tracking from Phase 5</x:v>
+      </x:c>
+      <x:c r="E30" s="15" t="str">
+        <x:v>Phase 5/PHASE5_DEV_HANDOFF.md</x:v>
+      </x:c>
+      <x:c r="F30" s="15" t="str">
+        <x:v>BA decision 2026-07-28</x:v>
+      </x:c>
+      <x:c r="G30" s="15" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="H30" s="22" t="str">
+        <x:v>Future Backlog</x:v>
+      </x:c>
+      <x:c r="I30" s="15" t="str">
+        <x:v>BA/PO</x:v>
+      </x:c>
+      <x:c r="J30" s="74" t="n">
+        <x:v>46231</x:v>
+      </x:c>
+      <x:c r="K30" s="74" t="n">
+        <x:v>46231</x:v>
+      </x:c>
+      <x:c r="L30" s="15" t="str">
+        <x:v>No Release Tracking implementation is claimed; future observation may be proposed under Reports</x:v>
+      </x:c>
+      <x:c r="M30" s="15" t="str">
+        <x:v>Future Reports proposal</x:v>
+      </x:c>
+      <x:c r="N30" s="15" t="str">
+        <x:v>Supersedes the prior P5.3 selected-Release screen proposal</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="54" customHeight="1">
@@ -3198,7 +3153,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H31" s="28" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I31" s="15" t="str">
         <x:v>BA/PO</x:v>
@@ -3206,60 +3161,66 @@
       <x:c r="J31" s="74" t="n">
         <x:v>46229</x:v>
       </x:c>
-      <x:c r="K31" s="74"/>
+      <x:c r="K31" s="74" t="n">
+        <x:v>46231</x:v>
+      </x:c>
       <x:c r="L31" s="15" t="str">
-        <x:v>Plan list, create modal, Teams by Total, allocations, publish and RBAC pass UAT</x:v>
+        <x:v>Single-Release Team capacity planning, allocations, metrics, warnings and publish lifecycle are BA accepted</x:v>
       </x:c>
       <x:c r="M31" s="15" t="str">
-        <x:v>Docs alignment -&gt; CAP-1 mockup</x:v>
+        <x:v>DEV handoff</x:v>
       </x:c>
       <x:c r="N31" s="15" t="str">
-        <x:v>BA confirmed 2026-07-26: Rally child Projects map to Mini Rally Teams; one Draft/Published plan per Project+Release</x:v>
+        <x:v>P5.2 closed 2026-07-28; production persistence/API/server authorization remains DEV scope</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="54" customHeight="1">
       <x:c r="A32" s="15" t="str">
-        <x:v>BA-0503</x:v>
+        <x:v>BA-F503</x:v>
       </x:c>
       <x:c r="B32" s="15" t="str">
         <x:v>Phase 5</x:v>
       </x:c>
       <x:c r="C32" s="15" t="str">
-        <x:v>Release Tracking</x:v>
+        <x:v>Reports Observation</x:v>
       </x:c>
       <x:c r="D32" s="15" t="str">
-        <x:v>Define and accept Release KPI and Feature progress tracking</x:v>
+        <x:v>Preserve Reports as the preferred future cross-release observation direction</x:v>
       </x:c>
       <x:c r="E32" s="15" t="str">
-        <x:v>Phase 5/03_Release_Tracking/SRS.md</x:v>
+        <x:v>Future_Backlog</x:v>
       </x:c>
       <x:c r="F32" s="15" t="str">
-        <x:v>BA-0502</x:v>
+        <x:v>Phase 5 close decision</x:v>
       </x:c>
       <x:c r="G32" s="15" t="str">
-        <x:v>P0</x:v>
+        <x:v>P2</x:v>
       </x:c>
       <x:c r="H32" s="25" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Future Backlog</x:v>
       </x:c>
       <x:c r="I32" s="15" t="str">
         <x:v>BA/PO</x:v>
       </x:c>
-      <x:c r="J32" s="74"/>
-      <x:c r="K32" s="74"/>
+      <x:c r="J32" s="74" t="n">
+        <x:v>46231</x:v>
+      </x:c>
+      <x:c r="K32" s="74" t="n">
+        <x:v>46231</x:v>
+      </x:c>
       <x:c r="L32" s="15" t="str">
-        <x:v>Plan Estimate rollup, zero-estimate handling and no auto Release state pass UAT</x:v>
+        <x:v>Phase 5 close does not define or claim a Report feature</x:v>
       </x:c>
       <x:c r="M32" s="15" t="str">
-        <x:v>Feature proposal</x:v>
+        <x:v>Future feature proposal</x:v>
       </x:c>
       <x:c r="N32" s="15" t="str">
-        <x:v>Starts after P5.2 Capacity Planning closes</x:v>
+        <x:v>Requires separate proposal, SRS, confirmation and delivery gates</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="54" customHeight="1">
       <x:c r="A33" s="57" t="str">
-        <x:v>BA-0504</x:v>
+        <x:v>BA-0503</x:v>
       </x:c>
       <x:c r="B33" s="57" t="str">
         <x:v>Phase 5</x:v>
@@ -3271,74 +3232,74 @@
         <x:v>Close Phase 5 and publish the dedicated DEV handoff</x:v>
       </x:c>
       <x:c r="E33" s="57" t="str">
-        <x:v>Phase 5 test pack + traceability + Phase 5 DEV handoff</x:v>
+        <x:v>Phase 5/PHASE5_DEV_HANDOFF.md</x:v>
       </x:c>
       <x:c r="F33" s="57" t="str">
-        <x:v>BA-0501..0503</x:v>
+        <x:v>BA-0501 + BA-0502 + scope decision</x:v>
       </x:c>
       <x:c r="G33" s="57" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H33" s="59" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I33" s="57" t="str">
         <x:v>BA/UAT</x:v>
       </x:c>
-      <x:c r="J33" s="75"/>
-      <x:c r="K33" s="75"/>
+      <x:c r="J33" s="75" t="n">
+        <x:v>46231</x:v>
+      </x:c>
+      <x:c r="K33" s="75" t="n">
+        <x:v>46231</x:v>
+      </x:c>
       <x:c r="L33" s="57" t="str">
-        <x:v>P5.1-P5.3 closed; build/runtime/test evidence complete; BA accepts phase</x:v>
+        <x:v>P5.1/P5.2 closed; Release Tracking excluded; documents/workbook/test disposition aligned</x:v>
       </x:c>
       <x:c r="M33" s="57" t="str">
-        <x:v>DEV handoff</x:v>
+        <x:v>Developer document review</x:v>
       </x:c>
       <x:c r="N33" s="57" t="str">
-        <x:v>Handoff is created only after Phase 5 close</x:v>
+        <x:v>Phase 5 is BA/mockup closed and DEV handoff ready; production implementation is not started</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="54" customHeight="1">
       <x:c r="A34" s="57" t="str">
-        <x:v>BA-0505</x:v>
+        <x:v>BA-F504</x:v>
       </x:c>
       <x:c r="B34" s="57" t="str">
         <x:v>Future</x:v>
       </x:c>
       <x:c r="C34" s="57" t="str">
-        <x:v>Release Planning</x:v>
+        <x:v>Preliminary Estimate Config</x:v>
       </x:c>
       <x:c r="D34" s="57" t="str">
-        <x:v>Keep Release Planning deferred until BA re-promotes it</x:v>
+        <x:v>Define user-managed Preliminary Estimate point/count mapping</x:v>
       </x:c>
       <x:c r="E34" s="57" t="str">
-        <x:v>Future_Backlog/02_Release_Planning.md</x:v>
+        <x:v>Future_Backlog</x:v>
       </x:c>
       <x:c r="F34" s="57" t="str">
-        <x:v>BA decision 2026-07-26</x:v>
+        <x:v>Project Management design proposal</x:v>
       </x:c>
       <x:c r="G34" s="57" t="str">
         <x:v>P2</x:v>
       </x:c>
       <x:c r="H34" s="61" t="str">
-        <x:v>Done</x:v>
+        <x:v>Future Backlog</x:v>
       </x:c>
       <x:c r="I34" s="57" t="str">
         <x:v>BA/PO</x:v>
       </x:c>
-      <x:c r="J34" s="75" t="n">
-        <x:v>46229</x:v>
-      </x:c>
-      <x:c r="K34" s="75" t="n">
-        <x:v>46229</x:v>
-      </x:c>
+      <x:c r="J34" s="75"/>
+      <x:c r="K34" s="75"/>
       <x:c r="L34" s="57" t="str">
-        <x:v>Active Phase 5 order no longer depends on Release Planning</x:v>
+        <x:v>Production does not silently treat the mock mapping as a permanent hard-coded rule</x:v>
       </x:c>
       <x:c r="M34" s="57" t="str">
         <x:v>Future backlog review</x:v>
       </x:c>
       <x:c r="N34" s="57" t="str">
-        <x:v>Capacity Planning publish is the active Phase 5 assignment mechanism</x:v>
+        <x:v>Confirmed future location: Settings &gt; Workspace &gt; Project Management</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5211,45 +5172,33 @@
       <x:c r="N31" s="15" t="str"/>
     </x:row>
     <x:row r="32" ht="54" customHeight="1">
-      <x:c r="A32" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DEV-0501</x:t>
-        </x:is>
+      <x:c r="A32" s="15" t="str">
+        <x:v>DEV-0501</x:v>
       </x:c>
       <x:c r="B32" s="15" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Phase 5</x:t>
         </x:is>
       </x:c>
-      <x:c r="C32" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Portfolio Items</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D32" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implement production Portfolio Items from the closed Phase 5 handoff</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E32" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Future Phase 5 DEV handoff</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F32" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BA-0501 + Phase 5 close</x:t>
-        </x:is>
+      <x:c r="C32" s="15" t="str">
+        <x:v>Portfolio Items</x:v>
+      </x:c>
+      <x:c r="D32" s="15" t="str">
+        <x:v>Implement production Portfolio Items from the closed Phase 5 handoff</x:v>
+      </x:c>
+      <x:c r="E32" s="15" t="str">
+        <x:v>Phase 5/PHASE5_DEV_HANDOFF.md</x:v>
+      </x:c>
+      <x:c r="F32" s="15" t="str">
+        <x:v>BA-0501 + Phase 5 close</x:v>
       </x:c>
       <x:c r="G32" s="15" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">P0</x:t>
         </x:is>
       </x:c>
-      <x:c r="H32" s="34" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Needs BA</x:t>
-        </x:is>
+      <x:c r="H32" s="34" t="str">
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="I32" s="15" t="inlineStr">
         <x:is>
@@ -5258,170 +5207,120 @@
       </x:c>
       <x:c r="J32" s="74" t="n"/>
       <x:c r="K32" s="74" t="n"/>
-      <x:c r="L32" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Project-scoped RBAC, Feature data, Archive and rollups pass DevInt</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M32" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DevInt</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N32" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mockup implementation is not production authorization</x:t>
-        </x:is>
+      <x:c r="L32" s="15" t="str">
+        <x:v>Epic/Feature persistence, project scope, archive and leaf rollups pass DevInt</x:v>
+      </x:c>
+      <x:c r="M32" s="15" t="str">
+        <x:v>DevInt</x:v>
+      </x:c>
+      <x:c r="N32" s="15" t="str">
+        <x:v>Mockup acceptance is not production evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="54" customHeight="1">
-      <x:c r="A33" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DEV-0502</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B33" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phase 5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C33" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Release Planning</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D33" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implement Feature-to-Release planning</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E33" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Future Phase 5 DEV handoff</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F33" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DEV-0501 + BA-0502</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G33" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H33" s="34" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Needs BA</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I33" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FE DEV</x:t>
-        </x:is>
+      <x:c r="A33" s="15" t="str">
+        <x:v>DEV-F501</x:v>
+      </x:c>
+      <x:c r="B33" s="15" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="C33" s="15" t="str">
+        <x:v>Release Planning</x:v>
+      </x:c>
+      <x:c r="D33" s="15" t="str">
+        <x:v>Do not implement until BA re-promotes Release Planning</x:v>
+      </x:c>
+      <x:c r="E33" s="15" t="str">
+        <x:v>Future_Backlog</x:v>
+      </x:c>
+      <x:c r="F33" s="15" t="str">
+        <x:v>PO approval</x:v>
+      </x:c>
+      <x:c r="G33" s="15" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="H33" s="34" t="str">
+        <x:v>Future Backlog</x:v>
+      </x:c>
+      <x:c r="I33" s="15" t="str">
+        <x:v>DEV</x:v>
       </x:c>
       <x:c r="J33" s="74" t="n"/>
       <x:c r="K33" s="74" t="n"/>
-      <x:c r="L33" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Assign/move/unassign is project-scoped and does not duplicate Release CRUD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M33" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DevInt</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N33" s="15" t="n"/>
+      <x:c r="L33" s="15" t="str">
+        <x:v>No hidden or partial Release Planning implementation enters active navigation</x:v>
+      </x:c>
+      <x:c r="M33" s="15" t="str">
+        <x:v>Future backlog review</x:v>
+      </x:c>
+      <x:c r="N33" s="15" t="str">
+        <x:v>Excluded from closed Phase 5</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="54" customHeight="1">
-      <x:c r="A34" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DEV-0503</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B34" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phase 5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C34" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Release Tracking</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D34" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implement Release KPI and Feature progress tracking</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E34" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Future Phase 5 DEV handoff</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F34" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DEV-0502 + BA-0503</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G34" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H34" s="34" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Needs BA</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I34" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FE DEV</x:t>
-        </x:is>
+      <x:c r="A34" s="15" t="str">
+        <x:v>DEV-F502</x:v>
+      </x:c>
+      <x:c r="B34" s="15" t="str">
+        <x:v>Future</x:v>
+      </x:c>
+      <x:c r="C34" s="15" t="str">
+        <x:v>Release Tracking</x:v>
+      </x:c>
+      <x:c r="D34" s="15" t="str">
+        <x:v>Do not implement a dedicated Release Tracking screen from historical Phase 5 stubs</x:v>
+      </x:c>
+      <x:c r="E34" s="15" t="str">
+        <x:v>Future_Backlog</x:v>
+      </x:c>
+      <x:c r="F34" s="15" t="str">
+        <x:v>PO approval</x:v>
+      </x:c>
+      <x:c r="G34" s="15" t="str">
+        <x:v>P3</x:v>
+      </x:c>
+      <x:c r="H34" s="34" t="str">
+        <x:v>Future Backlog</x:v>
+      </x:c>
+      <x:c r="I34" s="15" t="str">
+        <x:v>DEV</x:v>
       </x:c>
       <x:c r="J34" s="74" t="n"/>
       <x:c r="K34" s="74" t="n"/>
-      <x:c r="L34" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Confirmed rollup, zero-state and manual Release lifecycle pass DevInt</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M34" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DevInt</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N34" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No fabricated burnup history</x:t>
-        </x:is>
+      <x:c r="L34" s="15" t="str">
+        <x:v>Future observation is proposed under Reports only after BA confirmation</x:v>
+      </x:c>
+      <x:c r="M34" s="15" t="str">
+        <x:v>Future backlog review</x:v>
+      </x:c>
+      <x:c r="N34" s="15" t="str">
+        <x:v>Removed from Phase 5 by BA 2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="54" customHeight="1">
       <x:c r="A35" s="15" t="str">
-        <x:v>DEV-0501</x:v>
+        <x:v>DEV-0502</x:v>
       </x:c>
       <x:c r="B35" s="15" t="str">
         <x:v>Phase 5</x:v>
       </x:c>
       <x:c r="C35" s="15" t="str">
-        <x:v>Portfolio Items</x:v>
+        <x:v>Portfolio Integration</x:v>
       </x:c>
       <x:c r="D35" s="15" t="str">
-        <x:v>Implement production Portfolio Items from the closed Phase 5 handoff</x:v>
+        <x:v>Integrate Epic/Feature identity and leaf rollups with Work Item, Backlog, Iteration and Task flows</x:v>
       </x:c>
       <x:c r="E35" s="15" t="str">
-        <x:v>Future Phase 5 DEV handoff</x:v>
+        <x:v>Phase 5/PHASE5_DEV_HANDOFF.md</x:v>
       </x:c>
       <x:c r="F35" s="15" t="str">
-        <x:v>BA-0501 + Phase 5 close</x:v>
+        <x:v>DEV-0501</x:v>
       </x:c>
       <x:c r="G35" s="15" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H35" s="28" t="str">
-        <x:v>Needs BA</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="I35" s="15" t="str">
         <x:v>FE DEV</x:v>
@@ -5429,18 +5328,18 @@
       <x:c r="J35" s="74"/>
       <x:c r="K35" s="74"/>
       <x:c r="L35" s="15" t="str">
-        <x:v>Project-scoped RBAC, Feature data, Archive and rollups pass DevInt</x:v>
+        <x:v>One shared record model drives every surface and cross-project links are rejected</x:v>
       </x:c>
       <x:c r="M35" s="15" t="str">
         <x:v>DevInt</x:v>
       </x:c>
       <x:c r="N35" s="15" t="str">
-        <x:v>Mockup implementation is not production authorization</x:v>
+        <x:v>Includes Feature field, Unscheduled Backlog behavior and shared Task hour rules</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="54" customHeight="1">
       <x:c r="A36" s="15" t="str">
-        <x:v>DEV-0502</x:v>
+        <x:v>DEV-0503</x:v>
       </x:c>
       <x:c r="B36" s="15" t="str">
         <x:v>Phase 5</x:v>
@@ -5449,19 +5348,19 @@
         <x:v>Capacity Planning</x:v>
       </x:c>
       <x:c r="D36" s="15" t="str">
-        <x:v>Implement single-Release Team capacity planning</x:v>
+        <x:v>Implement production single-Release Team capacity planning</x:v>
       </x:c>
       <x:c r="E36" s="15" t="str">
-        <x:v>Future Phase 5 DEV handoff</x:v>
+        <x:v>Phase 5/PHASE5_DEV_HANDOFF.md</x:v>
       </x:c>
       <x:c r="F36" s="15" t="str">
-        <x:v>DEV-0501 + BA-0502</x:v>
+        <x:v>DEV-0501 + Timebox Release registry</x:v>
       </x:c>
       <x:c r="G36" s="15" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H36" s="28" t="str">
-        <x:v>Needs BA</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="I36" s="15" t="str">
         <x:v>FE DEV</x:v>
@@ -5469,58 +5368,58 @@
       <x:c r="J36" s="74"/>
       <x:c r="K36" s="74"/>
       <x:c r="L36" s="15" t="str">
-        <x:v>Plan list/detail, Team capacity, allocations, publish and RBAC pass DevInt</x:v>
+        <x:v>Plan lifecycle, Team capacity, split allocations, metrics, warnings and publish pass DevInt</x:v>
       </x:c>
       <x:c r="M36" s="15" t="str">
         <x:v>DevInt</x:v>
       </x:c>
       <x:c r="N36" s="15" t="str">
-        <x:v>Publish updates Feature Release/Team only; no child Story/Defect cascade</x:v>
+        <x:v>Publish may update Feature Release/planned dates only; never Project/Team or child Story/Defect</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="54" customHeight="1">
       <x:c r="A37" s="15" t="str">
-        <x:v>DEV-0503</x:v>
+        <x:v>DEV-0504</x:v>
       </x:c>
       <x:c r="B37" s="15" t="str">
         <x:v>Phase 5</x:v>
       </x:c>
       <x:c r="C37" s="15" t="str">
-        <x:v>Release Tracking</x:v>
+        <x:v>Authorization</x:v>
       </x:c>
       <x:c r="D37" s="15" t="str">
-        <x:v>Implement Release KPI and Feature progress tracking</x:v>
+        <x:v>Enforce Portfolio and Capacity Project/Team scope plus temporary planner Full/View server-side</x:v>
       </x:c>
       <x:c r="E37" s="15" t="str">
-        <x:v>Future Phase 5 DEV handoff</x:v>
+        <x:v>Phase 5/PHASE5_DEV_HANDOFF.md</x:v>
       </x:c>
       <x:c r="F37" s="15" t="str">
-        <x:v>DEV-0502 + BA-0503</x:v>
+        <x:v>DEV-0501 + DEV-0503 + Phase 4 RBAC</x:v>
       </x:c>
       <x:c r="G37" s="15" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H37" s="25" t="str">
-        <x:v>Needs BA</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="I37" s="15" t="str">
-        <x:v>FE DEV</x:v>
+        <x:v>FE/BE DEV</x:v>
       </x:c>
       <x:c r="J37" s="74"/>
       <x:c r="K37" s="74"/>
       <x:c r="L37" s="15" t="str">
-        <x:v>Confirmed rollup, zero-state and manual Release lifecycle pass DevInt</x:v>
+        <x:v>Workspace Admin, managed/unmanaged Project Admin and Project Member negative paths pass</x:v>
       </x:c>
       <x:c r="M37" s="15" t="str">
-        <x:v>DevInt</x:v>
+        <x:v>Security/DevInt</x:v>
       </x:c>
       <x:c r="N37" s="15" t="str">
-        <x:v>No fabricated burnup history</x:v>
+        <x:v>Control visibility is not authorization evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="54" customHeight="1">
       <x:c r="A38" s="57" t="str">
-        <x:v>DEV-0504</x:v>
+        <x:v>DEV-0505</x:v>
       </x:c>
       <x:c r="B38" s="57" t="str">
         <x:v>Phase 5</x:v>
@@ -5529,19 +5428,19 @@
         <x:v>Regression</x:v>
       </x:c>
       <x:c r="D38" s="57" t="str">
-        <x:v>Add Phase 5 FE/component/E2E and authorization coverage</x:v>
+        <x:v>Add Phase 5 service/component/E2E and authorization coverage</x:v>
       </x:c>
       <x:c r="E38" s="57" t="str">
-        <x:v>Phase 5 test scenarios + future DEV handoff</x:v>
+        <x:v>Phase 5 test scenarios + PHASE5_DEV_HANDOFF.md</x:v>
       </x:c>
       <x:c r="F38" s="57" t="str">
-        <x:v>DEV-0501..0503</x:v>
+        <x:v>DEV-0501..0504</x:v>
       </x:c>
       <x:c r="G38" s="57" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="H38" s="59" t="str">
-        <x:v>Needs BA</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="I38" s="57" t="str">
         <x:v>DEV/QA</x:v>
@@ -5549,12 +5448,14 @@
       <x:c r="J38" s="75"/>
       <x:c r="K38" s="75"/>
       <x:c r="L38" s="57" t="str">
-        <x:v>Portfolio critical path and role/project negative cases pass</x:v>
+        <x:v>Portfolio/Capacity critical, negative, publish and cross-module regression paths pass</x:v>
       </x:c>
       <x:c r="M38" s="57" t="str">
         <x:v>UAT sign-off</x:v>
       </x:c>
-      <x:c r="N38" s="57"/>
+      <x:c r="N38" s="57" t="str">
+        <x:v>Historical Not Run/Partial mockup cases are required production acceptance coverage</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="54" customHeight="1">
       <x:c r="A39" s="57" t="str">
@@ -5567,7 +5468,7 @@
         <x:v>Deferred UI</x:v>
       </x:c>
       <x:c r="D39" s="57" t="str">
-        <x:v>Do not build Team/Iteration boards, generic Reports, Theme/Initiative, Release Planning, burnup history or multi-Release scenarios until prioritized</x:v>
+        <x:v>Do not build Team/Iteration boards, Reports, Release Planning, Release Tracking, Theme/deeper hierarchy, burnup history or multi-Release scenarios until prioritized</x:v>
       </x:c>
       <x:c r="E39" s="57" t="str">
         <x:v>Future_Backlog</x:v>
@@ -6195,25 +6096,23 @@
           <x:t xml:space="preserve">D-015</x:t>
         </x:is>
       </x:c>
-      <x:c r="B19" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Release Navigation</x:t>
-        </x:is>
+      <x:c r="B19" s="15" t="str">
+        <x:v>Release Tracking</x:v>
       </x:c>
       <x:c r="C19" s="15" t="str">
-        <x:v>Promoted to Phase 5 P5.3 after Capacity Planning; use Plan Estimate progress, separate zero-estimate items, no automatic Release state and no burnup until trustworthy history exists</x:v>
+        <x:v>Dedicated Release Tracking is removed from closed Phase 5; future cross-release observation should be proposed under Reports</x:v>
       </x:c>
       <x:c r="D19" s="19" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="E19" s="15" t="str">
-        <x:v>Phase 5</x:v>
+        <x:v>Future</x:v>
       </x:c>
       <x:c r="F19" s="15" t="str">
         <x:v>BA/PO</x:v>
       </x:c>
       <x:c r="G19" s="15" t="str">
-        <x:v>P5-GOV v2</x:v>
+        <x:v>P5-GOV v4 / BA decision 2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
@@ -6222,10 +6121,8 @@
           <x:t xml:space="preserve">D-016</x:t>
         </x:is>
       </x:c>
-      <x:c r="B20" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Release Tracking</x:t>
-        </x:is>
+      <x:c r="B20" s="15" t="str">
+        <x:v>Plan Dates</x:v>
       </x:c>
       <x:c r="C20" s="15" t="str">
         <x:v>Dates after 2026-07-26 in this workbook are proposed execution dates and may be re-baselined by BA/DEV leads</x:v>
@@ -6249,13 +6146,11 @@
           <x:t xml:space="preserve">D-017</x:t>
         </x:is>
       </x:c>
-      <x:c r="B21" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Plan Dates</x:t>
-        </x:is>
+      <x:c r="B21" s="15" t="str">
+        <x:v>Phase 5 Scope</x:v>
       </x:c>
       <x:c r="C21" s="15" t="str">
-        <x:v>Phase 5 active MVP is Portfolio Items, Capacity Planning and Release Tracking; Release Planning is Future Backlog</x:v>
+        <x:v>Closed Phase 5 MVP is Portfolio Items plus Capacity Planning; Release Planning/Tracking are excluded and Reports remain Future Backlog</x:v>
       </x:c>
       <x:c r="D21" s="19" t="str">
         <x:v>Confirmed</x:v>
@@ -6267,7 +6162,7 @@
         <x:v>BA/PO</x:v>
       </x:c>
       <x:c r="G21" s="15" t="str">
-        <x:v>P5-GOV v2</x:v>
+        <x:v>P5-GOV v4</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="54" customHeight="1">
@@ -6276,13 +6171,11 @@
           <x:t xml:space="preserve">D-018</x:t>
         </x:is>
       </x:c>
-      <x:c r="B22" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phase 5 Scope</x:t>
-        </x:is>
+      <x:c r="B22" s="57" t="str">
+        <x:v>Phase 5 Order</x:v>
       </x:c>
       <x:c r="C22" s="57" t="str">
-        <x:v>Execute P5.1 Portfolio Items -&gt; P5.2 Capacity Planning -&gt; P5.3 Release Tracking -&gt; P5.4 Phase closeout and DEV handoff</x:v>
+        <x:v>P5.1 Portfolio Items -&gt; P5.2 Capacity Planning -&gt; P5.3 scope removal -&gt; P5.4 phase closeout and DEV handoff</x:v>
       </x:c>
       <x:c r="D22" s="64" t="str">
         <x:v>Confirmed</x:v>
@@ -6294,7 +6187,7 @@
         <x:v>BA/DEV</x:v>
       </x:c>
       <x:c r="G22" s="57" t="str">
-        <x:v>P5-GOV v2</x:v>
+        <x:v>P5-GOV v4</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -6303,25 +6196,23 @@
           <x:t xml:space="preserve">D-019</x:t>
         </x:is>
       </x:c>
-      <x:c r="B23" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phase 5 Order</x:t>
-        </x:is>
+      <x:c r="B23" s="57" t="str">
+        <x:v>Phase 5 Readiness</x:v>
       </x:c>
       <x:c r="C23" s="57" t="str">
-        <x:v>P5.1 is BA accepted and closed for BA/mockup scope; production implementation waits for Phase 5 DEV handoff</x:v>
+        <x:v>P5.1 and P5.2 are BA accepted; production implementation may start from the dedicated Phase 5 DEV handoff</x:v>
       </x:c>
       <x:c r="D23" s="64" t="str">
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="E23" s="57" t="str">
-        <x:v>P5.1</x:v>
+        <x:v>Phase 5</x:v>
       </x:c>
       <x:c r="F23" s="57" t="str">
-        <x:v>BA</x:v>
+        <x:v>BA/DEV</x:v>
       </x:c>
       <x:c r="G23" s="57" t="str">
-        <x:v>P5.1 closure 2026-07-26</x:v>
+        <x:v>Phase 5 close 2026-07-28</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
@@ -6342,13 +6233,13 @@
         <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="E24" s="57" t="str">
-        <x:v>P5.1-P5.3</x:v>
+        <x:v>P5.1-P5.2</x:v>
       </x:c>
       <x:c r="F24" s="57" t="str">
         <x:v>BA/DEV</x:v>
       </x:c>
       <x:c r="G24" s="57" t="str">
-        <x:v>P5-GOV v2</x:v>
+        <x:v>P5-GOV v4</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="54" customHeight="1">
@@ -6384,10 +6275,8 @@
           <x:t xml:space="preserve">D-022</x:t>
         </x:is>
       </x:c>
-      <x:c r="B26" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Feature Archive</x:t>
-        </x:is>
+      <x:c r="B26" s="57" t="str">
+        <x:v>Release Planning</x:v>
       </x:c>
       <x:c r="C26" s="57" t="str">
         <x:v>Release Planning is deferred; Capacity Planning publish is the active Feature Release/Team assignment mechanism for Phase 5</x:v>
@@ -6411,25 +6300,23 @@
           <x:t xml:space="preserve">D-023</x:t>
         </x:is>
       </x:c>
-      <x:c r="B27" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Release Planning</x:t>
-        </x:is>
+      <x:c r="B27" s="57" t="str">
+        <x:v>Release Tracking</x:v>
       </x:c>
       <x:c r="C27" s="57" t="str">
-        <x:v>Use KPI + Feature list, Plan Estimate progress, separate zero-estimate items and no automatic Release transition</x:v>
+        <x:v>Historical selected-Release KPI/burnup proposals are superseded and do not authorize implementation</x:v>
       </x:c>
       <x:c r="D27" s="64" t="str">
-        <x:v>Confirmed</x:v>
+        <x:v>Superseded</x:v>
       </x:c>
       <x:c r="E27" s="57" t="str">
-        <x:v>P5.3</x:v>
+        <x:v>Future</x:v>
       </x:c>
       <x:c r="F27" s="57" t="str">
         <x:v>BA/DEV</x:v>
       </x:c>
       <x:c r="G27" s="57" t="str">
-        <x:v>P5-GOV v2</x:v>
+        <x:v>P5-GOV v4</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="54" customHeight="1">
@@ -6438,10 +6325,8 @@
           <x:t xml:space="preserve">D-024</x:t>
         </x:is>
       </x:c>
-      <x:c r="B28" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Release Tracking</x:t>
-        </x:is>
+      <x:c r="B28" s="57" t="str">
+        <x:v>Capacity Planning</x:v>
       </x:c>
       <x:c r="C28" s="57" t="str">
         <x:v>Capacity Planning uses Team rows, manual capacity, Draft/Published lifecycle, Project+Release uniqueness, single-Team Feature allocation and Publish to master Feature</x:v>
@@ -6465,10 +6350,8 @@
           <x:t xml:space="preserve">D-025</x:t>
         </x:is>
       </x:c>
-      <x:c r="B29" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Capacity Planning</x:t>
-        </x:is>
+      <x:c r="B29" s="57" t="str">
+        <x:v>Phase Gate</x:v>
       </x:c>
       <x:c r="C29" s="57" t="str">
         <x:v>Each feature requires proposal, BA confirmation, docs, implementation, verification and BA acceptance; create DEV handoff only after Phase 5 closes</x:v>
@@ -6483,7 +6366,7 @@
         <x:v>BA/DEV/QA</x:v>
       </x:c>
       <x:c r="G29" s="57" t="str">
-        <x:v>P5-GOV v2</x:v>
+        <x:v>P5-GOV v4</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
@@ -6492,35 +6375,23 @@
           <x:t xml:space="preserve">D-026</x:t>
         </x:is>
       </x:c>
-      <x:c r="B30" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phase Gate</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C30" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Each feature requires proposal, BA confirmation, docs, implementation, verification and BA acceptance; create DEV handoff only after Phase 5 closes</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D30" s="64" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Confirmed</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E30" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Phase 5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F30" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BA/DEV/QA</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G30" s="57" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P5-GOV v1</x:t>
-        </x:is>
+      <x:c r="B30" s="57" t="str">
+        <x:v>Phase Gate</x:v>
+      </x:c>
+      <x:c r="C30" s="57" t="str">
+        <x:v>Phase 5 is BA/mockup closed and has a dedicated DEV handoff; future rule changes still require proposal, confirmation, docs, implementation and acceptance</x:v>
+      </x:c>
+      <x:c r="D30" s="64" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="E30" s="57" t="str">
+        <x:v>Phase 5</x:v>
+      </x:c>
+      <x:c r="F30" s="57" t="str">
+        <x:v>BA/DEV/QA</x:v>
+      </x:c>
+      <x:c r="G30" s="57" t="str">
+        <x:v>PHASE5_DEV_HANDOFF.md</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="40.5" customHeight="1">

</xml_diff>